<commit_message>
feat(rescate): editor «Datos del periodo» y recorridos J1-J6 en navegador real
- Editor tipo Excel en el expediente: movimientos, saldos iniciales,
  inventario, nómina, activos fijos (y ajustes/conteo si hay); agregar,
  duplicar, borrar, pegar desde Excel, cuentas del PUC, validación en vivo,
  guardado y recálculo al dejar de escribir, deshacer, archivos del periodo.
- Subir sin pasos extra: si no hay nada que decidir se calcula solo.
- Facturas DIAN: la subida reconoce de quién es el reporte (NIT y nombre).
- Playwright (frontend/e2e): J1 entrar, J2 subir (caso completo y DIAN),
  J3 navegar, J4 editar cliente y socios, J5 editar valores, J6 descargas
  y datos para editar. Servidor aislado con base temporal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demo/dian/facturas_emitidas_enero_2025.xlsx
+++ b/docs/demo/dian/facturas_emitidas_enero_2025.xlsx
@@ -586,7 +586,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2f8ee9b4e2ca936e2c8c4f1713e8fdc47bc98d930ee5e48fa581610244dc761f6bf186196d7abed0bd1a6607d39180b3</t>
+          <t>b3a8fea82517ab43b7394c9bf3e48c85f6581443afa56a3d143b6a9159d8c72ed489b1528c4f8671c9f918e73662dd61</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -624,7 +624,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>901234567</t>
+          <t>901777888</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>879b909be2d1802578bce618e64d9f7088655badfe342e14e1adb8cbb9c9f4b31130286379f331607d162f45da45741b</t>
+          <t>18be39ddc5adc72ee1b47cb09c627079e7a582eaeb9d6992072dc8628d871a2e5bd3950dfe8c59f6be634bbc340d1390</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -750,7 +750,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>901234567</t>
+          <t>901777888</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>5ce93df16cd7f61638d08e25996a084671136da55d83ecb726e93508b19755568d94af347352394051c264ca02650f0e</t>
+          <t>bb7852582d79332df86137dca61ddf8aa3413558bf8cfc15f0e4053833bf780440dbf24bfceb70599022773f52509bca</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -876,7 +876,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>901234567</t>
+          <t>901777888</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ad45072c743ce37f921e5fccdd3dbd40b0440e1d785ca125d799f986f496eadfa8018ff5c1044a55cad088ad5f022a14</t>
+          <t>59a72b4ca2079d33d4d662414a78ef1fe3eb7784747d2fb4e16a8a63e52a39ef8b224ae32593d49385cf853644b31b54</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>901234567</t>
+          <t>901777888</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>b682b2d3913675f58fb5976e22a290d89a837fbfea7e330e41f857f80895238d34006cd14fd1108c31647cb8f22ff265</t>
+          <t>94cf4b50d1c41ae7499e87e230383c0f1f05bf1831da99c5a6ca4f4d862385bd813b663d2d426504005e39315102d6f7</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>901234567</t>
+          <t>901777888</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>879b909be2d1802578bce618e64d9f7088655badfe342e14e1adb8cbb9c9f4b31130286379f331607d162f45da45741b</t>
+          <t>18be39ddc5adc72ee1b47cb09c627079e7a582eaeb9d6992072dc8628d871a2e5bd3950dfe8c59f6be634bbc340d1390</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>901234567</t>
+          <t>901777888</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">

</xml_diff>